<commit_message>
chore: remove juan add ivan
</commit_message>
<xml_diff>
--- a/public/data/info.xlsx
+++ b/public/data/info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\cisdeli\Purdue\CiampittiLab\ciampitti-lab.github.io\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD7D56A7-DBBB-421C-9B21-E90A98FDE59D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD89A817-64E8-4256-A07A-50BDC5FBDC29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{680A29BD-E113-4DFE-A325-D924D35BBF8F}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="28800" windowHeight="15345" xr2:uid="{680A29BD-E113-4DFE-A325-D924D35BBF8F}"/>
   </bookViews>
   <sheets>
     <sheet name="team" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="156">
   <si>
     <t>role</t>
   </si>
@@ -497,19 +497,16 @@
     <t>juan_fiore.png</t>
   </si>
   <si>
-    <t>Juan Douglas</t>
-  </si>
-  <si>
-    <t>juan_douglas.jpg</t>
-  </si>
-  <si>
     <t>Agronomist graduated from the National University of Córdoba. Focused on digital agriculture with experience in Python and programming for agricultural applications. Areas of contribution include data management, digital tools, and the integration of technology into agricultural systems.</t>
   </si>
   <si>
-    <t>Agronomical Engineering undergraduate student from the national university of Colombia, passionate and skilled in fertigation, irrigation, soil physics, and the use of data in agriculture</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/juan-camilo-douglas-bolano-157646293/</t>
+    <t>ivan_mejia.jpg</t>
+  </si>
+  <si>
+    <t>Data Science student at Universidad del Norte (Barranquilla, Colombia). Focused on leveraging data analysis and processing tools using Python for knowledge extraction. Passionate about using data-driven solutions to solve real-world problems and improve people's quality of life through the advancement of digital agriculture.</t>
+  </si>
+  <si>
+    <t>Ivan Ramirez</t>
   </si>
 </sst>
 </file>
@@ -1088,19 +1085,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>152</v>
+        <v>14</v>
       </c>
       <c r="C10" t="s">
         <v>3</v>
       </c>
       <c r="D10" t="s">
-        <v>153</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>156</v>
+        <v>104</v>
       </c>
       <c r="F10" t="s">
-        <v>155</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1108,13 +1102,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="C11" t="s">
         <v>3</v>
       </c>
       <c r="D11" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F11" t="s">
         <v>154</v>
@@ -1145,16 +1139,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
+        <v>139</v>
       </c>
       <c r="C13" t="s">
         <v>3</v>
       </c>
       <c r="D13" t="s">
-        <v>104</v>
+        <v>151</v>
       </c>
       <c r="F13" t="s">
-        <v>32</v>
+        <v>152</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1243,7 +1237,6 @@
     <hyperlink ref="E15" r:id="rId5" xr:uid="{D4CFB1C7-1AE1-491B-850A-B6BFAE8BB6A7}"/>
     <hyperlink ref="E12" r:id="rId6" tooltip="https://www.linkedin.com/in/jjola-unal/" xr:uid="{9B18B642-568C-42D5-8EB7-C9BF52A122A6}"/>
     <hyperlink ref="E17" r:id="rId7" xr:uid="{83DA2968-3BAC-44C7-87DD-D7D2815CABF1}"/>
-    <hyperlink ref="E10" r:id="rId8" xr:uid="{C20D33EE-D7E5-4CF8-918D-658532FE0616}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update priscilas bio
</commit_message>
<xml_diff>
--- a/public/data/info.xlsx
+++ b/public/data/info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\cisdeli\Purdue\CiampittiLab\ciampitti-lab.github.io\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD89A817-64E8-4256-A07A-50BDC5FBDC29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1915EC92-F081-4C47-BD04-14ACBCE3CEC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="28800" windowHeight="15345" xr2:uid="{680A29BD-E113-4DFE-A325-D924D35BBF8F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{680A29BD-E113-4DFE-A325-D924D35BBF8F}"/>
   </bookViews>
   <sheets>
     <sheet name="team" sheetId="1" r:id="rId1"/>
@@ -371,9 +371,6 @@
     <t>pedro_cisdeli.jpg</t>
   </si>
   <si>
-    <t>Combining expertise in agronomy, remote sensing &amp; geographic information systems, and economics. Current research efforts are directed toward the sustainable intensification of agricultural systems and digital agriculture.</t>
-  </si>
-  <si>
     <t>hello_world.md</t>
   </si>
   <si>
@@ -507,6 +504,9 @@
   </si>
   <si>
     <t>Ivan Ramirez</t>
+  </si>
+  <si>
+    <t>Agronomist researching cropping systems and farmer decision-making, integrating remote sensing and digital agriculture to evaluate how technological innovation and environmental variability influence agricultural sustainability and productivity.</t>
   </si>
 </sst>
 </file>
@@ -893,14 +893,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87EB64B1-8415-484E-B4A1-A632CC3BB222}">
   <dimension ref="A1:F17"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="61.375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="182.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.8984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.3984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="61.3984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="182.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1020,7 +1020,7 @@
         <v>39</v>
       </c>
       <c r="F6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1060,7 +1060,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="28.5">
+    <row r="9" spans="1:6" ht="27.6">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1077,7 +1077,7 @@
         <v>41</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>110</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1102,16 +1102,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C11" t="s">
         <v>3</v>
       </c>
       <c r="D11" t="s">
+        <v>152</v>
+      </c>
+      <c r="F11" t="s">
         <v>153</v>
-      </c>
-      <c r="F11" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1119,19 +1119,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C12" t="s">
         <v>3</v>
       </c>
       <c r="D12" t="s">
+        <v>139</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>141</v>
-      </c>
       <c r="F12" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1139,16 +1139,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C13" t="s">
         <v>3</v>
       </c>
       <c r="D13" t="s">
+        <v>150</v>
+      </c>
+      <c r="F13" t="s">
         <v>151</v>
-      </c>
-      <c r="F13" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1156,16 +1156,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C14" t="s">
         <v>3</v>
       </c>
       <c r="D14" t="s">
+        <v>148</v>
+      </c>
+      <c r="F14" t="s">
         <v>149</v>
-      </c>
-      <c r="F14" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -1173,19 +1173,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C15" t="s">
         <v>3</v>
       </c>
       <c r="D15" t="s">
+        <v>118</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F15" t="s">
         <v>119</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="F15" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1213,19 +1213,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C17" t="s">
         <v>3</v>
       </c>
       <c r="D17" t="s">
+        <v>145</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>147</v>
-      </c>
       <c r="F17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -1245,12 +1245,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8353AB8B-5FB3-4C2E-B56B-5EAF5DE5DE00}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="3" max="3" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.8984375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1261,7 +1261,7 @@
         <v>17</v>
       </c>
       <c r="C1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D1" t="s">
         <v>18</v>
@@ -1284,25 +1284,25 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F2" t="s">
         <v>114</v>
       </c>
-      <c r="C2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D2" t="s">
-        <v>113</v>
-      </c>
-      <c r="E2" t="s">
-        <v>116</v>
-      </c>
-      <c r="F2" t="s">
-        <v>115</v>
-      </c>
       <c r="G2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H2" t="s">
         <v>111</v>
-      </c>
-      <c r="H2" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1310,25 +1310,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C3" t="s">
+        <v>132</v>
+      </c>
+      <c r="D3" t="s">
         <v>137</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>133</v>
       </c>
-      <c r="D3" t="s">
-        <v>138</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
+        <v>114</v>
+      </c>
+      <c r="G3" t="s">
         <v>134</v>
       </c>
-      <c r="F3" t="s">
-        <v>115</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>135</v>
-      </c>
-      <c r="H3" t="s">
-        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -1339,7 +1339,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA036B15-B04C-4846-822B-68722C1605FF}">
   <dimension ref="A1:G14"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="4" max="4" width="30" bestFit="1" customWidth="1"/>
   </cols>
@@ -1625,22 +1625,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>120</v>
+      </c>
+      <c r="C13" t="s">
         <v>121</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>122</v>
-      </c>
-      <c r="D13" t="s">
-        <v>123</v>
       </c>
       <c r="E13">
         <v>2025</v>
       </c>
       <c r="F13" t="s">
+        <v>123</v>
+      </c>
+      <c r="G13" t="s">
         <v>124</v>
-      </c>
-      <c r="G13" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -1648,19 +1648,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>126</v>
+      </c>
+      <c r="C14" t="s">
         <v>127</v>
       </c>
-      <c r="C14" t="s">
-        <v>128</v>
-      </c>
       <c r="D14" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E14">
         <v>2025</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G14" s="1"/>
     </row>

</xml_diff>

<commit_message>
chore: update me to a phd
</commit_message>
<xml_diff>
--- a/public/data/info.xlsx
+++ b/public/data/info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\cisdeli\Purdue\CiampittiLab\ciampitti-lab.github.io\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1915EC92-F081-4C47-BD04-14ACBCE3CEC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{786D0E22-F118-4614-AEAE-13588A6BE334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{680A29BD-E113-4DFE-A325-D924D35BBF8F}"/>
   </bookViews>
@@ -39,12 +39,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="155">
   <si>
     <t>role</t>
-  </si>
-  <si>
-    <t>MSc. Student</t>
   </si>
   <si>
     <t>PhD. Student</t>
@@ -905,22 +902,22 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
       </c>
       <c r="D1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -928,19 +925,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" t="s">
         <v>43</v>
-      </c>
-      <c r="D2" t="s">
-        <v>99</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="F2" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -954,13 +951,13 @@
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>109</v>
-      </c>
-      <c r="E3" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E3" t="s">
         <v>36</v>
       </c>
       <c r="F3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -971,16 +968,16 @@
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>100</v>
-      </c>
-      <c r="E4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>27</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -991,16 +988,16 @@
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>103</v>
-      </c>
-      <c r="E5" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E5" t="s">
         <v>38</v>
       </c>
       <c r="F5" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1008,19 +1005,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>105</v>
-      </c>
-      <c r="E6" t="s">
-        <v>39</v>
+        <v>108</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="F6" t="s">
-        <v>116</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1028,36 +1025,36 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="23.4" customHeight="1">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="27.6">
@@ -1065,19 +1062,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1085,16 +1082,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1102,16 +1099,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C11" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D11" t="s">
+        <v>151</v>
+      </c>
+      <c r="F11" t="s">
         <v>152</v>
-      </c>
-      <c r="F11" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1119,19 +1116,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>140</v>
+      </c>
+      <c r="C12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" t="s">
+        <v>138</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="F12" t="s">
         <v>141</v>
-      </c>
-      <c r="C12" t="s">
-        <v>3</v>
-      </c>
-      <c r="D12" t="s">
-        <v>139</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="F12" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1139,16 +1136,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C13" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D13" t="s">
+        <v>149</v>
+      </c>
+      <c r="F13" t="s">
         <v>150</v>
-      </c>
-      <c r="F13" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1156,16 +1153,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>146</v>
+      </c>
+      <c r="C14" t="s">
+        <v>2</v>
+      </c>
+      <c r="D14" t="s">
         <v>147</v>
       </c>
-      <c r="C14" t="s">
-        <v>3</v>
-      </c>
-      <c r="D14" t="s">
+      <c r="F14" t="s">
         <v>148</v>
-      </c>
-      <c r="F14" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -1173,19 +1170,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
+        <v>116</v>
+      </c>
+      <c r="C15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D15" t="s">
         <v>117</v>
       </c>
-      <c r="C15" t="s">
-        <v>3</v>
-      </c>
-      <c r="D15" t="s">
+      <c r="E15" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F15" t="s">
         <v>118</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="F15" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1193,19 +1190,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C16" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1213,26 +1210,26 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
+        <v>142</v>
+      </c>
+      <c r="C17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="F17" t="s">
         <v>143</v>
-      </c>
-      <c r="C17" t="s">
-        <v>3</v>
-      </c>
-      <c r="D17" t="s">
-        <v>145</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="F17" t="s">
-        <v>144</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E3" r:id="rId1" xr:uid="{AAA55F43-9F3C-40DB-9B47-46AAC432FF09}"/>
+    <hyperlink ref="E6" r:id="rId1" xr:uid="{AAA55F43-9F3C-40DB-9B47-46AAC432FF09}"/>
     <hyperlink ref="E2" r:id="rId2" xr:uid="{A94255E5-8ECE-483E-BE8F-EE9B37DAE260}"/>
-    <hyperlink ref="E5" r:id="rId3" xr:uid="{F9808E56-71B8-4EF9-927B-9D68DAE7673D}"/>
+    <hyperlink ref="E4" r:id="rId3" xr:uid="{F9808E56-71B8-4EF9-927B-9D68DAE7673D}"/>
     <hyperlink ref="E8" r:id="rId4" xr:uid="{2A6658AF-7FC0-4FB5-9A94-14DD4D416741}"/>
     <hyperlink ref="E15" r:id="rId5" xr:uid="{D4CFB1C7-1AE1-491B-850A-B6BFAE8BB6A7}"/>
     <hyperlink ref="E12" r:id="rId6" tooltip="https://www.linkedin.com/in/jjola-unal/" xr:uid="{9B18B642-568C-42D5-8EB7-C9BF52A122A6}"/>
@@ -1255,28 +1252,28 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>129</v>
+      </c>
+      <c r="D1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
-        <v>130</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>18</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H1" t="s">
         <v>19</v>
-      </c>
-      <c r="F1" t="s">
-        <v>45</v>
-      </c>
-      <c r="G1" t="s">
-        <v>46</v>
-      </c>
-      <c r="H1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -1284,25 +1281,25 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E2" t="s">
+        <v>114</v>
+      </c>
+      <c r="F2" t="s">
         <v>113</v>
       </c>
-      <c r="C2" t="s">
-        <v>131</v>
-      </c>
-      <c r="D2" t="s">
-        <v>112</v>
-      </c>
-      <c r="E2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F2" t="s">
-        <v>114</v>
-      </c>
       <c r="G2" t="s">
+        <v>109</v>
+      </c>
+      <c r="H2" t="s">
         <v>110</v>
-      </c>
-      <c r="H2" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1310,25 +1307,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>135</v>
+      </c>
+      <c r="C3" t="s">
+        <v>131</v>
+      </c>
+      <c r="D3" t="s">
         <v>136</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>132</v>
       </c>
-      <c r="D3" t="s">
-        <v>137</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
+        <v>113</v>
+      </c>
+      <c r="G3" t="s">
         <v>133</v>
       </c>
-      <c r="F3" t="s">
-        <v>114</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>134</v>
-      </c>
-      <c r="H3" t="s">
-        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -1346,25 +1343,25 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
-        <v>17</v>
-      </c>
       <c r="C1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" t="s">
         <v>21</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" t="s">
         <v>22</v>
       </c>
-      <c r="E1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>23</v>
-      </c>
-      <c r="G1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -1372,22 +1369,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" t="s">
         <v>47</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>48</v>
-      </c>
-      <c r="D2" t="s">
-        <v>49</v>
       </c>
       <c r="E2">
         <v>2025</v>
       </c>
       <c r="F2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -1395,22 +1392,22 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3" t="s">
         <v>52</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>53</v>
-      </c>
-      <c r="D3" t="s">
-        <v>54</v>
       </c>
       <c r="E3">
         <v>2025</v>
       </c>
       <c r="F3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G3" t="s">
         <v>55</v>
-      </c>
-      <c r="G3" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -1418,22 +1415,22 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" t="s">
         <v>57</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>58</v>
-      </c>
-      <c r="D4" t="s">
-        <v>59</v>
       </c>
       <c r="E4">
         <v>2025</v>
       </c>
       <c r="F4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -1441,22 +1438,22 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" t="s">
         <v>62</v>
       </c>
-      <c r="C5" t="s">
-        <v>63</v>
-      </c>
       <c r="D5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E5">
         <v>2025</v>
       </c>
       <c r="F5" t="s">
+        <v>63</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -1464,22 +1461,22 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" t="s">
         <v>66</v>
       </c>
-      <c r="C6" t="s">
-        <v>67</v>
-      </c>
       <c r="D6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E6">
         <v>2025</v>
       </c>
       <c r="F6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -1487,22 +1484,22 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D7" t="s">
         <v>72</v>
-      </c>
-      <c r="C7" t="s">
-        <v>71</v>
-      </c>
-      <c r="D7" t="s">
-        <v>73</v>
       </c>
       <c r="E7">
         <v>2025</v>
       </c>
       <c r="F7" t="s">
+        <v>73</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -1510,22 +1507,22 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C8" t="s">
         <v>76</v>
       </c>
-      <c r="C8" t="s">
-        <v>77</v>
-      </c>
       <c r="D8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E8">
         <v>2025</v>
       </c>
       <c r="F8" t="s">
+        <v>77</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -1533,22 +1530,22 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C9" t="s">
         <v>80</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>81</v>
-      </c>
-      <c r="D9" t="s">
-        <v>82</v>
       </c>
       <c r="E9">
         <v>2025</v>
       </c>
       <c r="F9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -1556,22 +1553,22 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C10" t="s">
         <v>85</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>86</v>
-      </c>
-      <c r="D10" t="s">
-        <v>87</v>
       </c>
       <c r="E10">
         <v>2025</v>
       </c>
       <c r="F10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -1579,22 +1576,22 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C11" t="s">
         <v>88</v>
       </c>
-      <c r="C11" t="s">
-        <v>89</v>
-      </c>
       <c r="D11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E11">
         <v>2025</v>
       </c>
       <c r="F11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -1602,22 +1599,22 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C12" t="s">
         <v>90</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>91</v>
-      </c>
-      <c r="D12" t="s">
-        <v>92</v>
       </c>
       <c r="E12">
         <v>2025</v>
       </c>
       <c r="F12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -1625,22 +1622,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>119</v>
+      </c>
+      <c r="C13" t="s">
         <v>120</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>121</v>
-      </c>
-      <c r="D13" t="s">
-        <v>122</v>
       </c>
       <c r="E13">
         <v>2025</v>
       </c>
       <c r="F13" t="s">
+        <v>122</v>
+      </c>
+      <c r="G13" t="s">
         <v>123</v>
-      </c>
-      <c r="G13" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -1648,19 +1645,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>125</v>
+      </c>
+      <c r="C14" t="s">
         <v>126</v>
       </c>
-      <c r="C14" t="s">
-        <v>127</v>
-      </c>
       <c r="D14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E14">
         <v>2025</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G14" s="1"/>
     </row>

</xml_diff>

<commit_message>
chore: update leo and jorge
</commit_message>
<xml_diff>
--- a/public/data/info.xlsx
+++ b/public/data/info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\cisdeli\Purdue\CiampittiLab\ciampitti-lab.github.io\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{786D0E22-F118-4614-AEAE-13588A6BE334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4D8E85F-B0B9-4FDA-95A3-CE905E667F0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{680A29BD-E113-4DFE-A325-D924D35BBF8F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{680A29BD-E113-4DFE-A325-D924D35BBF8F}"/>
   </bookViews>
   <sheets>
     <sheet name="team" sheetId="1" r:id="rId1"/>
@@ -362,9 +362,6 @@
     <t>priscila_cano.jpg</t>
   </si>
   <si>
-    <t>Agronomist developing decision support models for precision nitrogen management in corn. Integrates crop physiology, sensing technologies, and statistics to improve productivity while reducing environmental impact.</t>
-  </si>
-  <si>
     <t>pedro_cisdeli.jpg</t>
   </si>
   <si>
@@ -504,6 +501,9 @@
   </si>
   <si>
     <t>Agronomist researching cropping systems and farmer decision-making, integrating remote sensing and digital agriculture to evaluate how technological innovation and environmental variability influence agricultural sustainability and productivity.</t>
+  </si>
+  <si>
+    <t>Agronomist focused on precision nitrogen management in corn through crop physiology, sensing technologies, and data-driven approaches.</t>
   </si>
 </sst>
 </file>
@@ -890,14 +890,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87EB64B1-8415-484E-B4A1-A632CC3BB222}">
   <dimension ref="A1:F17"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.59765625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.8984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.3984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="61.3984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="182.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="61.375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="182.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -977,7 +977,7 @@
         <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>107</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -997,7 +997,7 @@
         <v>38</v>
       </c>
       <c r="F5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1011,7 +1011,7 @@
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>35</v>
@@ -1037,7 +1037,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="23.4" customHeight="1">
+    <row r="8" spans="1:6" ht="23.45" customHeight="1">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1057,7 +1057,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="27.6">
+    <row r="9" spans="1:6" ht="28.5">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1074,7 +1074,7 @@
         <v>40</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1099,16 +1099,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C11" t="s">
         <v>2</v>
       </c>
       <c r="D11" t="s">
+        <v>150</v>
+      </c>
+      <c r="F11" t="s">
         <v>151</v>
-      </c>
-      <c r="F11" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1116,19 +1116,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C12" t="s">
         <v>2</v>
       </c>
       <c r="D12" t="s">
+        <v>137</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>139</v>
-      </c>
       <c r="F12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1136,16 +1136,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C13" t="s">
         <v>2</v>
       </c>
       <c r="D13" t="s">
+        <v>148</v>
+      </c>
+      <c r="F13" t="s">
         <v>149</v>
-      </c>
-      <c r="F13" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1153,16 +1153,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C14" t="s">
         <v>2</v>
       </c>
       <c r="D14" t="s">
+        <v>146</v>
+      </c>
+      <c r="F14" t="s">
         <v>147</v>
-      </c>
-      <c r="F14" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -1170,19 +1170,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C15" t="s">
         <v>2</v>
       </c>
       <c r="D15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F15" t="s">
         <v>117</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="F15" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1210,19 +1210,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C17" t="s">
         <v>2</v>
       </c>
       <c r="D17" t="s">
+        <v>143</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>145</v>
-      </c>
       <c r="F17" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -1242,12 +1242,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8353AB8B-5FB3-4C2E-B56B-5EAF5DE5DE00}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="3" max="3" width="11.8984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.3984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1258,7 +1258,7 @@
         <v>16</v>
       </c>
       <c r="C1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D1" t="s">
         <v>17</v>
@@ -1281,25 +1281,25 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E2" t="s">
+        <v>113</v>
+      </c>
+      <c r="F2" t="s">
         <v>112</v>
       </c>
-      <c r="C2" t="s">
-        <v>130</v>
-      </c>
-      <c r="D2" t="s">
-        <v>111</v>
-      </c>
-      <c r="E2" t="s">
-        <v>114</v>
-      </c>
-      <c r="F2" t="s">
-        <v>113</v>
-      </c>
       <c r="G2" t="s">
+        <v>108</v>
+      </c>
+      <c r="H2" t="s">
         <v>109</v>
-      </c>
-      <c r="H2" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1307,25 +1307,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C3" t="s">
+        <v>130</v>
+      </c>
+      <c r="D3" t="s">
         <v>135</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>131</v>
       </c>
-      <c r="D3" t="s">
-        <v>136</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
+        <v>112</v>
+      </c>
+      <c r="G3" t="s">
         <v>132</v>
       </c>
-      <c r="F3" t="s">
-        <v>113</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>133</v>
-      </c>
-      <c r="H3" t="s">
-        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -1336,7 +1336,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA036B15-B04C-4846-822B-68722C1605FF}">
   <dimension ref="A1:G14"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="4" max="4" width="30" bestFit="1" customWidth="1"/>
   </cols>
@@ -1622,22 +1622,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>118</v>
+      </c>
+      <c r="C13" t="s">
         <v>119</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>120</v>
-      </c>
-      <c r="D13" t="s">
-        <v>121</v>
       </c>
       <c r="E13">
         <v>2025</v>
       </c>
       <c r="F13" t="s">
+        <v>121</v>
+      </c>
+      <c r="G13" t="s">
         <v>122</v>
-      </c>
-      <c r="G13" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -1645,19 +1645,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>124</v>
+      </c>
+      <c r="C14" t="s">
         <v>125</v>
       </c>
-      <c r="C14" t="s">
-        <v>126</v>
-      </c>
       <c r="D14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E14">
         <v>2025</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G14" s="1"/>
     </row>

</xml_diff>